<commit_message>
Checked the data for fish species
</commit_message>
<xml_diff>
--- a/Data/Master/Fish species_Initial Check.xlsx
+++ b/Data/Master/Fish species_Initial Check.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/louwclaassens/Documents/WorldFish/Ikan Ba Futura_2023/Science and colabs/Ecological Modeling/Timor-Leste South Coast/Timor_South_Ecopath/Timor_Ecopath/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/louwclaassens/Documents/WorldFish/Ikan Ba Futura_2023/Science and colabs/Ecological Modeling/Timor-Leste South Coast/Timor_South_Ecopath/Timor_Ecopath/Data/Master/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D633117-A3F5-CA40-B25C-9DF13A3A09F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8485D58B-6AEA-E149-827F-712753CBC5A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="220" yWindow="680" windowWidth="28040" windowHeight="16780" xr2:uid="{8B661F92-5076-464D-8422-0F08A21EB7CC}"/>
   </bookViews>
@@ -2862,7 +2862,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42D43BBC-FD48-6D4B-B79D-D054E095EE14}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:R138"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
@@ -2939,7 +2938,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="119" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:17" ht="119" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
         <v>6</v>
       </c>
@@ -2990,7 +2989,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="3" spans="1:17" ht="85" hidden="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:17" ht="85" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
         <v>9</v>
       </c>
@@ -3037,7 +3036,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="68" hidden="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:17" ht="68" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
         <v>11</v>
       </c>
@@ -3086,7 +3085,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="5" spans="1:17" ht="17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:17" ht="17" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
         <v>9</v>
       </c>
@@ -3129,7 +3128,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="6" spans="1:17" ht="51" hidden="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:17" ht="51" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
         <v>13</v>
       </c>
@@ -3174,7 +3173,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="7" spans="1:17" ht="102" hidden="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:17" ht="102" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
         <v>17</v>
       </c>
@@ -3223,7 +3222,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="8" spans="1:17" ht="51" hidden="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:17" ht="51" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
         <v>17</v>
       </c>
@@ -3268,7 +3267,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="9" spans="1:17" ht="136" hidden="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:17" ht="136" x14ac:dyDescent="0.2">
       <c r="A9" s="17" t="s">
         <v>17</v>
       </c>
@@ -3317,7 +3316,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="10" spans="1:17" ht="51" hidden="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:17" ht="51" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
         <v>20</v>
       </c>
@@ -3362,7 +3361,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="11" spans="1:17" ht="68" hidden="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:17" ht="68" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
         <v>6</v>
       </c>
@@ -3409,7 +3408,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="12" spans="1:17" ht="17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:17" ht="17" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
         <v>6</v>
       </c>
@@ -3444,7 +3443,7 @@
       <c r="P12" s="6"/>
       <c r="Q12" s="6"/>
     </row>
-    <row r="13" spans="1:17" ht="102" hidden="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:17" ht="102" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
         <v>6</v>
       </c>
@@ -3493,7 +3492,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="14" spans="1:17" ht="68" hidden="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:17" ht="68" x14ac:dyDescent="0.2">
       <c r="A14" s="12" t="s">
         <v>6</v>
       </c>
@@ -3542,7 +3541,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="15" spans="1:17" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
         <v>6</v>
       </c>
@@ -3589,7 +3588,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="16" spans="1:17" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
         <v>6</v>
       </c>
@@ -3632,7 +3631,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="17" spans="1:17" ht="51" hidden="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:17" ht="51" x14ac:dyDescent="0.2">
       <c r="A17" s="17" t="s">
         <v>6</v>
       </c>
@@ -3683,7 +3682,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="18" spans="1:17" ht="17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:17" ht="17" x14ac:dyDescent="0.2">
       <c r="A18" s="5" t="s">
         <v>6</v>
       </c>
@@ -3718,7 +3717,7 @@
       <c r="P18" s="6"/>
       <c r="Q18" s="6"/>
     </row>
-    <row r="19" spans="1:17" ht="136" hidden="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:17" ht="136" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
         <v>6</v>
       </c>
@@ -3765,7 +3764,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="20" spans="1:17" ht="51" hidden="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:17" ht="51" x14ac:dyDescent="0.2">
       <c r="A20" s="5" t="s">
         <v>6</v>
       </c>
@@ -3861,7 +3860,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="22" spans="1:17" ht="68" hidden="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:17" ht="68" x14ac:dyDescent="0.2">
       <c r="A22" s="5" t="s">
         <v>6</v>
       </c>
@@ -3906,7 +3905,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="23" spans="1:17" ht="102" hidden="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:17" ht="102" x14ac:dyDescent="0.2">
       <c r="A23" s="5" t="s">
         <v>6</v>
       </c>
@@ -3955,7 +3954,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="24" spans="1:17" ht="85" hidden="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:17" ht="85" x14ac:dyDescent="0.2">
       <c r="A24" s="5" t="s">
         <v>6</v>
       </c>
@@ -4000,7 +3999,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="25" spans="1:17" ht="51" hidden="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:17" ht="51" x14ac:dyDescent="0.2">
       <c r="A25" s="5" t="s">
         <v>6</v>
       </c>
@@ -4047,7 +4046,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="26" spans="1:17" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A26" s="5" t="s">
         <v>6</v>
       </c>
@@ -4092,7 +4091,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="27" spans="1:17" ht="51" hidden="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:17" ht="51" x14ac:dyDescent="0.2">
       <c r="A27" s="19" t="s">
         <v>162</v>
       </c>
@@ -4137,7 +4136,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="28" spans="1:17" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A28" s="5" t="s">
         <v>6</v>
       </c>
@@ -4186,7 +4185,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="29" spans="1:17" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A29" s="5" t="s">
         <v>6</v>
       </c>
@@ -4231,7 +4230,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="30" spans="1:17" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A30" s="5" t="s">
         <v>6</v>
       </c>
@@ -4276,7 +4275,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="31" spans="1:17" ht="85" hidden="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:17" ht="85" x14ac:dyDescent="0.2">
       <c r="A31" s="5" t="s">
         <v>6</v>
       </c>
@@ -4323,7 +4322,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="32" spans="1:17" ht="17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:17" ht="17" x14ac:dyDescent="0.2">
       <c r="A32" s="5" t="s">
         <v>6</v>
       </c>
@@ -4366,7 +4365,7 @@
       <c r="P32" s="6"/>
       <c r="Q32" s="6"/>
     </row>
-    <row r="33" spans="1:17" ht="221" hidden="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:17" ht="221" x14ac:dyDescent="0.2">
       <c r="A33" s="5" t="s">
         <v>6</v>
       </c>
@@ -4415,7 +4414,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="34" spans="1:17" ht="204" hidden="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:17" ht="204" x14ac:dyDescent="0.2">
       <c r="A34" s="5" t="s">
         <v>6</v>
       </c>
@@ -4464,7 +4463,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="35" spans="1:17" ht="119" hidden="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:17" ht="119" x14ac:dyDescent="0.2">
       <c r="A35" s="5" t="s">
         <v>6</v>
       </c>
@@ -4513,7 +4512,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="36" spans="1:17" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A36" s="5" t="s">
         <v>6</v>
       </c>
@@ -4558,7 +4557,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="37" spans="1:17" ht="17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:17" ht="17" x14ac:dyDescent="0.2">
       <c r="A37" s="5" t="s">
         <v>6</v>
       </c>
@@ -4593,7 +4592,7 @@
       <c r="P37" s="6"/>
       <c r="Q37" s="6"/>
     </row>
-    <row r="38" spans="1:17" ht="85" hidden="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:17" ht="85" x14ac:dyDescent="0.2">
       <c r="A38" s="5" t="s">
         <v>6</v>
       </c>
@@ -4638,7 +4637,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="39" spans="1:17" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A39" s="5" t="s">
         <v>6</v>
       </c>
@@ -4683,7 +4682,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="40" spans="1:17" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A40" s="5" t="s">
         <v>6</v>
       </c>
@@ -4730,7 +4729,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="41" spans="1:17" ht="17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:17" ht="17" x14ac:dyDescent="0.2">
       <c r="A41" s="5" t="s">
         <v>51</v>
       </c>
@@ -4775,7 +4774,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="42" spans="1:17" ht="17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:17" ht="17" x14ac:dyDescent="0.2">
       <c r="A42" s="5" t="s">
         <v>51</v>
       </c>
@@ -4818,7 +4817,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="43" spans="1:17" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A43" s="5" t="s">
         <v>17</v>
       </c>
@@ -4865,7 +4864,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="44" spans="1:17" ht="68" hidden="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:17" ht="68" x14ac:dyDescent="0.2">
       <c r="A44" s="5" t="s">
         <v>17</v>
       </c>
@@ -4910,7 +4909,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="45" spans="1:17" ht="85" hidden="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:17" ht="85" x14ac:dyDescent="0.2">
       <c r="A45" s="5" t="s">
         <v>17</v>
       </c>
@@ -4957,7 +4956,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="46" spans="1:17" ht="102" hidden="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:17" ht="102" x14ac:dyDescent="0.2">
       <c r="A46" s="5" t="s">
         <v>57</v>
       </c>
@@ -5005,7 +5004,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="47" spans="1:17" ht="51" hidden="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:17" ht="51" x14ac:dyDescent="0.2">
       <c r="A47" s="5" t="s">
         <v>206</v>
       </c>
@@ -5056,7 +5055,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="48" spans="1:17" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A48" s="5" t="s">
         <v>59</v>
       </c>
@@ -5103,7 +5102,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="49" spans="1:17" ht="102" hidden="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:17" ht="102" x14ac:dyDescent="0.2">
       <c r="A49" s="5" t="s">
         <v>61</v>
       </c>
@@ -5156,7 +5155,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="50" spans="1:17" ht="119" hidden="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:17" ht="119" x14ac:dyDescent="0.2">
       <c r="A50" s="5" t="s">
         <v>63</v>
       </c>
@@ -5205,7 +5204,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="51" spans="1:17" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A51" s="5" t="s">
         <v>66</v>
       </c>
@@ -5256,7 +5255,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="52" spans="1:17" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A52" s="25" t="s">
         <v>67</v>
       </c>
@@ -5303,7 +5302,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="53" spans="1:17" ht="119" hidden="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:17" ht="119" x14ac:dyDescent="0.2">
       <c r="A53" s="5" t="s">
         <v>57</v>
       </c>
@@ -5348,7 +5347,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="54" spans="1:17" ht="68" hidden="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:17" ht="68" x14ac:dyDescent="0.2">
       <c r="A54" s="5" t="s">
         <v>71</v>
       </c>
@@ -5397,7 +5396,7 @@
       <c r="P54" s="16"/>
       <c r="Q54" s="16"/>
     </row>
-    <row r="55" spans="1:17" ht="136" hidden="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:17" ht="136" x14ac:dyDescent="0.2">
       <c r="A55" s="20" t="s">
         <v>72</v>
       </c>
@@ -5440,7 +5439,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="56" spans="1:17" ht="68" hidden="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:17" ht="68" x14ac:dyDescent="0.2">
       <c r="A56" s="5" t="s">
         <v>74</v>
       </c>
@@ -5491,7 +5490,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="57" spans="1:17" ht="51" hidden="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:17" ht="51" x14ac:dyDescent="0.2">
       <c r="A57" s="20" t="s">
         <v>76</v>
       </c>
@@ -5534,7 +5533,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="58" spans="1:17" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A58" s="5" t="s">
         <v>76</v>
       </c>
@@ -5579,7 +5578,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="59" spans="1:17" ht="51" hidden="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:17" ht="51" x14ac:dyDescent="0.2">
       <c r="A59" s="5" t="s">
         <v>79</v>
       </c>
@@ -5624,7 +5623,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="60" spans="1:17" ht="85" hidden="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:17" ht="85" x14ac:dyDescent="0.2">
       <c r="A60" s="5" t="s">
         <v>81</v>
       </c>
@@ -5671,7 +5670,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="61" spans="1:17" ht="17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:17" ht="17" x14ac:dyDescent="0.2">
       <c r="A61" s="5" t="s">
         <v>81</v>
       </c>
@@ -5714,7 +5713,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="62" spans="1:17" ht="17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:17" ht="17" x14ac:dyDescent="0.2">
       <c r="A62" s="5" t="s">
         <v>51</v>
       </c>
@@ -5757,7 +5756,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="63" spans="1:17" ht="170" hidden="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:17" ht="170" x14ac:dyDescent="0.2">
       <c r="A63" s="5" t="s">
         <v>84</v>
       </c>
@@ -5808,7 +5807,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="64" spans="1:17" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A64" s="20" t="s">
         <v>86</v>
       </c>
@@ -5851,7 +5850,7 @@
       <c r="P64" s="16"/>
       <c r="Q64" s="16"/>
     </row>
-    <row r="65" spans="1:17" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A65" s="5" t="s">
         <v>90</v>
       </c>
@@ -5896,7 +5895,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="66" spans="1:17" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A66" s="5" t="s">
         <v>90</v>
       </c>
@@ -5945,7 +5944,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="67" spans="1:17" ht="68" hidden="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:17" ht="68" x14ac:dyDescent="0.2">
       <c r="A67" s="5" t="s">
         <v>101</v>
       </c>
@@ -5992,7 +5991,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="68" spans="1:17" ht="51" hidden="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:17" ht="51" x14ac:dyDescent="0.2">
       <c r="A68" s="5" t="s">
         <v>393</v>
       </c>
@@ -6039,7 +6038,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="69" spans="1:17" ht="85" hidden="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:17" ht="85" x14ac:dyDescent="0.2">
       <c r="A69" s="5" t="s">
         <v>279</v>
       </c>
@@ -6082,7 +6081,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="70" spans="1:17" ht="51" hidden="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:17" ht="51" x14ac:dyDescent="0.2">
       <c r="A70" s="5" t="s">
         <v>281</v>
       </c>
@@ -6127,7 +6126,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="71" spans="1:17" ht="17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:17" ht="17" x14ac:dyDescent="0.2">
       <c r="A71" s="5" t="s">
         <v>283</v>
       </c>
@@ -6150,7 +6149,7 @@
       <c r="P71" s="6"/>
       <c r="Q71" s="6"/>
     </row>
-    <row r="72" spans="1:17" ht="102" hidden="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:17" ht="102" x14ac:dyDescent="0.2">
       <c r="A72" s="5" t="s">
         <v>284</v>
       </c>
@@ -6199,7 +6198,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="73" spans="1:17" ht="119" hidden="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:17" ht="119" x14ac:dyDescent="0.2">
       <c r="A73" s="5" t="s">
         <v>286</v>
       </c>
@@ -6244,7 +6243,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="74" spans="1:17" ht="17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:17" ht="17" x14ac:dyDescent="0.2">
       <c r="A74" s="5" t="s">
         <v>288</v>
       </c>
@@ -6281,7 +6280,7 @@
       <c r="P74" s="6"/>
       <c r="Q74" s="6"/>
     </row>
-    <row r="75" spans="1:17" ht="17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:17" ht="17" x14ac:dyDescent="0.2">
       <c r="A75" s="5" t="s">
         <v>290</v>
       </c>
@@ -6318,7 +6317,7 @@
       <c r="P75" s="6"/>
       <c r="Q75" s="6"/>
     </row>
-    <row r="76" spans="1:17" ht="102" hidden="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:17" ht="102" x14ac:dyDescent="0.2">
       <c r="A76" s="5" t="s">
         <v>292</v>
       </c>
@@ -6367,7 +6366,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="77" spans="1:17" ht="51" hidden="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:17" ht="51" x14ac:dyDescent="0.2">
       <c r="A77" s="5" t="s">
         <v>292</v>
       </c>
@@ -6414,7 +6413,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="78" spans="1:17" ht="221" hidden="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:17" ht="221" x14ac:dyDescent="0.2">
       <c r="A78" s="5" t="s">
         <v>86</v>
       </c>
@@ -6463,7 +6462,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="79" spans="1:17" ht="51" hidden="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:17" ht="51" x14ac:dyDescent="0.2">
       <c r="A79" s="5" t="s">
         <v>86</v>
       </c>
@@ -6509,7 +6508,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="80" spans="1:17" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A80" s="5" t="s">
         <v>297</v>
       </c>
@@ -6556,7 +6555,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="81" spans="1:17" ht="17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:17" ht="17" x14ac:dyDescent="0.2">
       <c r="A81" s="5" t="s">
         <v>299</v>
       </c>
@@ -6605,7 +6604,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="82" spans="1:17" ht="255" hidden="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:17" ht="255" x14ac:dyDescent="0.2">
       <c r="A82" s="6" t="s">
         <v>302</v>
       </c>
@@ -6654,7 +6653,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="83" spans="1:17" ht="51" hidden="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:17" ht="51" x14ac:dyDescent="0.2">
       <c r="A83" s="5" t="s">
         <v>303</v>
       </c>
@@ -6701,7 +6700,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="84" spans="1:17" ht="68" hidden="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:17" ht="68" x14ac:dyDescent="0.2">
       <c r="A84" s="5" t="s">
         <v>303</v>
       </c>
@@ -6746,7 +6745,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="85" spans="1:17" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A85" s="5" t="s">
         <v>306</v>
       </c>
@@ -6793,7 +6792,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="86" spans="1:17" ht="68" hidden="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:17" ht="68" x14ac:dyDescent="0.2">
       <c r="A86" s="5" t="s">
         <v>308</v>
       </c>
@@ -6842,7 +6841,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="87" spans="1:17" ht="153" hidden="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:17" ht="153" x14ac:dyDescent="0.2">
       <c r="A87" s="5" t="s">
         <v>310</v>
       </c>
@@ -6893,7 +6892,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="88" spans="1:17" ht="51" hidden="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:17" ht="51" x14ac:dyDescent="0.2">
       <c r="A88" s="6" t="s">
         <v>313</v>
       </c>
@@ -6938,7 +6937,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="89" spans="1:17" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A89" s="5" t="s">
         <v>313</v>
       </c>
@@ -6983,7 +6982,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="90" spans="1:17" ht="119" hidden="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:17" ht="119" x14ac:dyDescent="0.2">
       <c r="A90" s="32" t="s">
         <v>315</v>
       </c>
@@ -7030,7 +7029,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="91" spans="1:17" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A91" s="25" t="s">
         <v>317</v>
       </c>
@@ -7067,7 +7066,7 @@
       <c r="P91" s="6"/>
       <c r="Q91" s="6"/>
     </row>
-    <row r="92" spans="1:17" ht="51" hidden="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:17" ht="51" x14ac:dyDescent="0.2">
       <c r="A92" s="6" t="s">
         <v>323</v>
       </c>
@@ -7112,7 +7111,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="93" spans="1:17" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A93" s="5" t="s">
         <v>57</v>
       </c>
@@ -7155,7 +7154,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="94" spans="1:17" ht="17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:17" ht="17" x14ac:dyDescent="0.2">
       <c r="A94" s="5" t="s">
         <v>320</v>
       </c>
@@ -7197,7 +7196,7 @@
         <v>459</v>
       </c>
     </row>
-    <row r="95" spans="1:17" ht="17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:17" ht="17" x14ac:dyDescent="0.2">
       <c r="A95" s="32" t="s">
         <v>324</v>
       </c>
@@ -7234,7 +7233,7 @@
       <c r="P95" s="6"/>
       <c r="Q95" s="6"/>
     </row>
-    <row r="96" spans="1:17" ht="85" hidden="1" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:17" ht="85" x14ac:dyDescent="0.2">
       <c r="A96" s="32" t="s">
         <v>324</v>
       </c>
@@ -7277,7 +7276,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="97" spans="1:17" ht="68" hidden="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:17" ht="68" x14ac:dyDescent="0.2">
       <c r="A97" s="32" t="s">
         <v>327</v>
       </c>
@@ -7322,7 +7321,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="98" spans="1:17" ht="170" hidden="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:17" ht="170" x14ac:dyDescent="0.2">
       <c r="A98" s="32" t="s">
         <v>327</v>
       </c>
@@ -7367,7 +7366,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="99" spans="1:17" ht="136" hidden="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:17" ht="136" x14ac:dyDescent="0.2">
       <c r="A99" s="32" t="s">
         <v>329</v>
       </c>
@@ -7416,7 +7415,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="100" spans="1:17" ht="119" hidden="1" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:17" ht="119" x14ac:dyDescent="0.2">
       <c r="A100" s="32" t="s">
         <v>331</v>
       </c>
@@ -7461,7 +7460,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="101" spans="1:17" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A101" s="32" t="s">
         <v>333</v>
       </c>
@@ -7506,7 +7505,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="102" spans="1:17" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A102" s="32" t="s">
         <v>335</v>
       </c>
@@ -7553,7 +7552,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="103" spans="1:17" ht="119" hidden="1" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:17" ht="119" x14ac:dyDescent="0.2">
       <c r="A103" s="32" t="s">
         <v>337</v>
       </c>
@@ -7598,7 +7597,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="104" spans="1:17" ht="68" hidden="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:17" ht="68" x14ac:dyDescent="0.2">
       <c r="A104" s="32" t="s">
         <v>337</v>
       </c>
@@ -7645,7 +7644,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="105" spans="1:17" ht="153" hidden="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:17" ht="153" x14ac:dyDescent="0.2">
       <c r="A105" s="32" t="s">
         <v>337</v>
       </c>
@@ -7694,7 +7693,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="106" spans="1:17" ht="51" hidden="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:17" ht="51" x14ac:dyDescent="0.2">
       <c r="A106" s="32" t="s">
         <v>337</v>
       </c>
@@ -7737,7 +7736,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="107" spans="1:17" ht="119" hidden="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:17" ht="119" x14ac:dyDescent="0.2">
       <c r="A107" s="32" t="s">
         <v>343</v>
       </c>
@@ -7784,7 +7783,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="108" spans="1:17" ht="85" hidden="1" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:17" ht="85" x14ac:dyDescent="0.2">
       <c r="A108" s="32" t="s">
         <v>344</v>
       </c>
@@ -7831,7 +7830,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="109" spans="1:17" ht="51" hidden="1" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:17" ht="51" x14ac:dyDescent="0.2">
       <c r="A109" s="32" t="s">
         <v>346</v>
       </c>
@@ -7878,7 +7877,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="110" spans="1:17" ht="17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:17" ht="17" x14ac:dyDescent="0.2">
       <c r="A110" s="32" t="s">
         <v>346</v>
       </c>
@@ -7923,7 +7922,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="111" spans="1:17" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A111" s="32" t="s">
         <v>349</v>
       </c>
@@ -7970,7 +7969,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="112" spans="1:17" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A112" s="32" t="s">
         <v>350</v>
       </c>
@@ -8017,7 +8016,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="113" spans="1:17" ht="17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:17" ht="17" x14ac:dyDescent="0.2">
       <c r="A113" s="32" t="s">
         <v>350</v>
       </c>
@@ -8062,7 +8061,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="114" spans="1:17" ht="51" hidden="1" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:17" ht="51" x14ac:dyDescent="0.2">
       <c r="A114" s="32" t="s">
         <v>353</v>
       </c>
@@ -8105,7 +8104,7 @@
         <v>504</v>
       </c>
     </row>
-    <row r="115" spans="1:17" ht="17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:17" ht="17" x14ac:dyDescent="0.2">
       <c r="A115" s="32" t="s">
         <v>355</v>
       </c>
@@ -8148,7 +8147,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="116" spans="1:17" ht="17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:17" ht="17" x14ac:dyDescent="0.2">
       <c r="A116" s="32" t="s">
         <v>357</v>
       </c>
@@ -8185,7 +8184,7 @@
       <c r="P116" s="6"/>
       <c r="Q116" s="6"/>
     </row>
-    <row r="117" spans="1:17" ht="85" hidden="1" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:17" ht="85" x14ac:dyDescent="0.2">
       <c r="A117" s="31" t="s">
         <v>359</v>
       </c>
@@ -8232,7 +8231,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="118" spans="1:17" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A118" s="32" t="s">
         <v>361</v>
       </c>
@@ -8275,7 +8274,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="119" spans="1:17" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A119" s="32" t="s">
         <v>363</v>
       </c>
@@ -8322,7 +8321,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="120" spans="1:17" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A120" s="32" t="s">
         <v>365</v>
       </c>
@@ -8373,7 +8372,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="121" spans="1:17" ht="17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:17" ht="17" x14ac:dyDescent="0.2">
       <c r="A121" s="32" t="s">
         <v>367</v>
       </c>
@@ -8418,7 +8417,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="122" spans="1:17" ht="153" hidden="1" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:17" ht="153" x14ac:dyDescent="0.2">
       <c r="A122" s="32" t="s">
         <v>66</v>
       </c>
@@ -8469,7 +8468,7 @@
         <v>517</v>
       </c>
     </row>
-    <row r="123" spans="1:17" ht="85" hidden="1" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:17" ht="85" x14ac:dyDescent="0.2">
       <c r="A123" s="32" t="s">
         <v>370</v>
       </c>
@@ -8518,7 +8517,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="124" spans="1:17" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A124" s="32" t="s">
         <v>370</v>
       </c>
@@ -8565,7 +8564,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="125" spans="1:17" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A125" s="5" t="s">
         <v>437</v>
       </c>
@@ -8616,7 +8615,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="126" spans="1:17" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A126" s="5" t="s">
         <v>439</v>
       </c>
@@ -8667,7 +8666,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="127" spans="1:17" ht="17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:17" ht="17" x14ac:dyDescent="0.2">
       <c r="A127" s="5" t="s">
         <v>521</v>
       </c>
@@ -8701,7 +8700,7 @@
       <c r="P127" s="6"/>
       <c r="Q127" s="6"/>
     </row>
-    <row r="128" spans="1:17" ht="102" hidden="1" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:17" ht="102" x14ac:dyDescent="0.2">
       <c r="A128" s="5" t="s">
         <v>523</v>
       </c>
@@ -8744,7 +8743,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="129" spans="1:17" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:17" ht="34" x14ac:dyDescent="0.2">
       <c r="A129" s="5" t="s">
         <v>531</v>
       </c>
@@ -8789,7 +8788,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="130" spans="1:17" ht="153" hidden="1" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:17" ht="153" x14ac:dyDescent="0.2">
       <c r="A130" s="34" t="s">
         <v>393</v>
       </c>
@@ -8838,7 +8837,7 @@
         <v>543</v>
       </c>
     </row>
-    <row r="131" spans="1:17" ht="85" hidden="1" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:17" ht="85" x14ac:dyDescent="0.2">
       <c r="A131" s="34" t="s">
         <v>538</v>
       </c>
@@ -8927,13 +8926,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R131" xr:uid="{42D43BBC-FD48-6D4B-B79D-D054E095EE14}">
-    <filterColumn colId="9">
-      <filters>
-        <filter val="12844"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:R131" xr:uid="{42D43BBC-FD48-6D4B-B79D-D054E095EE14}"/>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>